<commit_message>
feat: planilha modelo em português + números no formato brasileiro
- Modelos XLSX e CSV com cabeçalhos em PT: SKU, Nome, Descrição, Marca,
  NCM, EAN, Peso (kg), Altura (cm), Largura (cm), Comprimento (cm),
  Imagens, Estoque
- Parser normaliza cabeçalhos (minúsculas, sem acentos, ignora sufixos
  como "(kg)") — aceita PT e EN, qualquer caixa; sinônimos: código,
  produto, fotos, quantidade
- Números no formato brasileiro: "1,5" → 1.5 e "1.234,56" → 1234.56
- Tela de importação lista as colunas em português

Testado: CSV PT, XLSX PT, CSV EN legado, cabeçalhos em CAIXA ALTA com
acento e decimais com vírgula.

https://claude.ai/code/session_014FBLrNetQrpRwJyYy69hpe
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/products-template.xlsx
+++ b/apps/web/public/templates/products-template.xlsx
@@ -13,40 +13,40 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
-    <t>sku</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>brand</t>
-  </si>
-  <si>
-    <t>ncm</t>
-  </si>
-  <si>
-    <t>gtin</t>
-  </si>
-  <si>
-    <t>weight</t>
-  </si>
-  <si>
-    <t>height</t>
-  </si>
-  <si>
-    <t>width</t>
-  </si>
-  <si>
-    <t>length</t>
-  </si>
-  <si>
-    <t>images</t>
-  </si>
-  <si>
-    <t>stock</t>
+    <t>SKU</t>
+  </si>
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
+    <t>Descrição</t>
+  </si>
+  <si>
+    <t>Marca</t>
+  </si>
+  <si>
+    <t>NCM</t>
+  </si>
+  <si>
+    <t>EAN</t>
+  </si>
+  <si>
+    <t>Peso (kg)</t>
+  </si>
+  <si>
+    <t>Altura (cm)</t>
+  </si>
+  <si>
+    <t>Largura (cm)</t>
+  </si>
+  <si>
+    <t>Comprimento (cm)</t>
+  </si>
+  <si>
+    <t>Imagens</t>
+  </si>
+  <si>
+    <t>Estoque</t>
   </si>
   <si>
     <t>PROD-001</t>
@@ -477,8 +477,10 @@
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="17" customWidth="1"/>
     <col min="11" max="11" width="40" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
   </cols>

</xml_diff>